<commit_message>
Update lab project materials and schedules
</commit_message>
<xml_diff>
--- a/generated_outputs/Weekly Schedules.xlsx
+++ b/generated_outputs/Weekly Schedules.xlsx
@@ -431,7 +431,7 @@
     <col width="80" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="49" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lab 1: Lab 1 in-lab activity</t>
+          <t>Lab 1: Completed `lab-starter.R` with the requested objects and plots. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -532,7 +532,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lab 2: Tutorial 2 hash | Lab 2 in-lab activity</t>
+          <t>Lab 2: Completed `lab-starter.R` with the fitted models and requested autograder objects. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Project1-1: Project 1 outline</t>
+          <t>Project1-1: Completed Project 1 outline submitted through the course platform. | Shared Google Doc containing the title, motivation, questions, data description, limitations, roles, and timeline.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -596,7 +596,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Project1-2: Project 1 plan</t>
+          <t>Project1-2: Project 1 progress materials submitted through the course platform. | Cleaned-data notes, initial EDA, revised questions, and accessible shared Google Doc link.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -628,7 +628,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Project1-3: Project 1 progress report</t>
+          <t>Project1-3: Project 1 progress report submitted through the course platform. | Candidate models, diagnostics, justified modeling direction, and accessible shared Google Doc link.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -660,7 +660,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Project1-4: Project 1 video</t>
+          <t>Project1-4: Project 1 final presentation materials or video submitted through the course platform. | Shared script/document link and reproducible supporting files.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Project2-1: Project 2 initial plan</t>
+          <t>Project2-1: Completed Project 2 outline submitted through the course platform. | Shared document with study plans, research questions, real-data plan, timeline, roles, and planned outputs.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Project2-2: Project 2 plan</t>
+          <t>Project2-2: Project 2 simulation-design materials submitted through the course platform. | Simulation algorithm, planned outputs, shared document link, and reproducible code files.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -756,7 +756,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Project2-3: Project 2 progress report</t>
+          <t>Project2-3: Project 2 progress report submitted through the course platform. | Real-data analysis, diagnostics, shared document link, and reproducible code files.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -784,7 +784,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Project2-4: Project 2 write-up</t>
+          <t>Project2-4: Project 2 writeup, code, and required supporting files submitted through the course platform. | Shared Google Doc link and confirmation of group review.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -816,7 +816,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lab 3: Tutorial 3 hash</t>
+          <t>Lab 3: Completed `lab-starter.R` with the required posterior objects. | Completed posterior-probability practice or Tutorial 3 hash, as assigned.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lab 4: Tutorial 4 hash</t>
+          <t>Lab 4: Completed `lab-starter.R` with the requested posterior summaries. | Completed conjugate-model practice or Tutorial 4 hash, as assigned.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lab 5: Tutorial 5 hash</t>
+          <t>Lab 5: Completed `lab-starter.R` with the data, log-posterior, credible interval, and posterior predictive mean objects. | Completed Bayesian-regression practice or Tutorial 5 hash, as assigned.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>

</xml_diff>

<commit_message>
Align skills-lab deliverables with the stated policy
Every skills lab now lists the same two deliverables: the tutorial hash
submitted before lab, and the in-lab response sheet after. This replaces
the inconsistent wording, where labs 1-2 listed only the response sheet
and labs 3-5 offered practice or a hash "as assigned".

Students do not submit lab-starter.R, so drop the Gradescope submission
line from the five starter scripts.

Applied to lab_summary.md and the five lab plan files, with the site
outputs regenerated to match.
</commit_message>
<xml_diff>
--- a/generated_outputs/Weekly Schedules.xlsx
+++ b/generated_outputs/Weekly Schedules.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lab 1: Completed `lab-starter.R` with the requested objects and plots. | Completed in-lab activity response sheet.</t>
+          <t>Lab 1: Tutorial 1 hash submitted before lab. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -532,7 +532,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lab 2: Completed `lab-starter.R` with the fitted models and requested autograder objects. | Completed in-lab activity response sheet.</t>
+          <t>Lab 2: Tutorial 2 hash submitted before lab. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -816,7 +816,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lab 3: Completed `lab-starter.R` with the required posterior objects. | Completed posterior-probability practice or Tutorial 3 hash, as assigned.</t>
+          <t>Lab 3: Tutorial 3 hash submitted before lab. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lab 4: Completed `lab-starter.R` with the requested posterior summaries. | Completed conjugate-model practice or Tutorial 4 hash, as assigned.</t>
+          <t>Lab 4: Tutorial 4 hash submitted before lab. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lab 5: Completed `lab-starter.R` with the data, log-posterior, credible interval, and posterior predictive mean objects. | Completed Bayesian-regression practice or Tutorial 5 hash, as assigned.</t>
+          <t>Lab 5: Tutorial 5 hash submitted before lab. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>

</xml_diff>

<commit_message>
Move deliverable deadlines to the week after each session
Deliverable dates were computed from the session's own week, so once the
deadline weekday moved to Tuesday it landed the day before the Wednesday
lab it belonged to. The response sheet is completed during that lab, so
every deadline was unmeetable.

Compute the date from the following week instead. All 13 deliverables
now fall six days after their session, and Lab 1 moves from its lab day
to Tuesday Sep 8.

Reword the hash line to "Tutorial N hash (due before lab)", since the
shared deadline is now after the lab even though the hash precedes it.
</commit_message>
<xml_diff>
--- a/generated_outputs/Weekly Schedules.xlsx
+++ b/generated_outputs/Weekly Schedules.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lab 1: Tutorial 1 hash submitted before lab. | Completed in-lab activity response sheet.</t>
+          <t>Lab 1: Tutorial 1 hash (due before lab). | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -532,7 +532,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lab 2: Tutorial 2 hash submitted before lab. | Completed in-lab activity response sheet.</t>
+          <t>Lab 2: Tutorial 2 hash (due before lab). | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -816,7 +816,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lab 3: Tutorial 3 hash submitted before lab. | Completed in-lab activity response sheet.</t>
+          <t>Lab 3: Tutorial 3 hash (due before lab). | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lab 4: Tutorial 4 hash submitted before lab. | Completed in-lab activity response sheet.</t>
+          <t>Lab 4: Tutorial 4 hash (due before lab). | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lab 5: Tutorial 5 hash submitted before lab. | Completed in-lab activity response sheet.</t>
+          <t>Lab 5: Tutorial 5 hash (due before lab). | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>

</xml_diff>

<commit_message>
Split the tutorial hash into its own deadline
The hash is due before its own lab and the worksheet after it, so a
single deliverable deadline could not express both. Deliverable lines
naming a tutorial hash now generate a separate earlier deadline.

Timing, per instructor:

- Tutorial hash: Tuesday, the day before its lab
- Worksheet: Wednesday, end of the lab day
- Lab 1: both collected the following Tuesday, since its tutorial cannot
  be due before the first lab of the term

Project deliverables get their own pattern row so that retiming lab
worksheets leaves the eight project milestones on their Tuesday. Rows
left out of the table inherit the lab deliverable settings.
</commit_message>
<xml_diff>
--- a/generated_outputs/Weekly Schedules.xlsx
+++ b/generated_outputs/Weekly Schedules.xlsx
@@ -500,7 +500,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lab 1: Tutorial 1 hash (due before lab). | Completed in-lab activity response sheet.</t>
+          <t>Lab 1: Tutorial 1 hash. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -532,7 +532,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lab 2: Tutorial 2 hash (due before lab). | Completed in-lab activity response sheet.</t>
+          <t>Lab 2: Tutorial 2 hash. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -816,7 +816,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lab 3: Tutorial 3 hash (due before lab). | Completed in-lab activity response sheet.</t>
+          <t>Lab 3: Tutorial 3 hash. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lab 4: Tutorial 4 hash (due before lab). | Completed in-lab activity response sheet.</t>
+          <t>Lab 4: Tutorial 4 hash. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lab 5: Tutorial 5 hash (due before lab). | Completed in-lab activity response sheet.</t>
+          <t>Lab 5: Tutorial 5 hash. | Completed in-lab activity response sheet.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>

</xml_diff>